<commit_message>
Add owner-contribution entry for cash expense and Dashboard bank check box
Logs the $23.48 USPS cash payment as Personal Money In on Funding so the
sheet's cash position reconciles exactly with the bank account. Adds a
Bank Check section to the Dashboard: expected bank balance vs. actual,
with a difference cell that turns green at $0 and red otherwise.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D2uQe8piQyqLuwZ6jefB1X
</commit_message>
<xml_diff>
--- a/BOYNT_Year1_Financial_Tracker.xlsx
+++ b/BOYNT_Year1_Financial_Tracker.xlsx
@@ -33,7 +33,7 @@
     <numFmt numFmtId="167" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="168" formatCode="mmm\ yyyy"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -160,8 +160,27 @@
       <color rgb="004A7A5E"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="001F3B57"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3B57"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="007F7F7F"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -218,6 +237,16 @@
         <fgColor rgb="00E4F7EC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E7D8C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCEEF3"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -260,7 +289,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -339,11 +368,18 @@
     <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="13" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="13" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="30">
+  <dxfs count="32">
     <dxf>
       <font>
         <b val="1"/>
@@ -625,6 +661,28 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="009C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2070,7 +2128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2387,6 +2445,93 @@
       <c r="F24" s="22">
         <f>IF(N(F23)=0,"",F21/F23)</f>
         <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="68" t="inlineStr">
+        <is>
+          <t>BANK CHECK — does the sheet match the bank?</t>
+        </is>
+      </c>
+      <c r="C27" s="69" t="n"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="70" t="inlineStr">
+        <is>
+          <t>Sheet cash position (auto)</t>
+        </is>
+      </c>
+      <c r="C28" s="71">
+        <f>C17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="70" t="inlineStr">
+        <is>
+          <t>Business cash in hand, not deposited</t>
+        </is>
+      </c>
+      <c r="C29" s="72" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="73" t="inlineStr">
+        <is>
+          <t>EXPECTED BANK BALANCE (auto)</t>
+        </is>
+      </c>
+      <c r="C30" s="71">
+        <f>C28-C29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="70" t="inlineStr">
+        <is>
+          <t>Your actual bank balance (type it in)</t>
+        </is>
+      </c>
+      <c r="C31" s="72" t="n"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="73" t="inlineStr">
+        <is>
+          <t>DIFFERENCE (should be $0)</t>
+        </is>
+      </c>
+      <c r="C32" s="72">
+        <f>IF(C31="","",C31-C30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="74" t="inlineStr">
+        <is>
+          <t>Rule of thumb: pay from the business account. If personal cash/card covers something,</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="74" t="inlineStr">
+        <is>
+          <t>log the expense AND a matching 'Personal Money In' on Funding. If the business gets</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="74" t="inlineStr">
+        <is>
+          <t>cash, deposit it (or list it in 'cash in hand' above until you do). Difference turns</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="74" t="inlineStr">
+        <is>
+          <t>green when the sheet and bank agree to the penny.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2416,6 +2561,14 @@
     </cfRule>
     <cfRule type="cellIs" priority="6" operator="lessThan" dxfId="0">
       <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C32">
+    <cfRule type="expression" priority="7" dxfId="30">
+      <formula>AND(C32&lt;&gt;"",ABS(C32)&lt;0.01)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="31">
+      <formula>AND(C32&lt;&gt;"",ABS(C32)&gt;=0.01)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7321,18 +7474,44 @@
       <c r="I22" s="9" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="35" t="n"/>
-      <c r="B23" s="9" t="n"/>
-      <c r="C23" s="9" t="n"/>
-      <c r="D23" s="9" t="n"/>
-      <c r="E23" s="54" t="n"/>
-      <c r="F23" s="54" t="n"/>
+      <c r="A23" s="35" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Personal Money In</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Zach (personal cash)</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Covered USPS box to Jack with personal cash</t>
+        </is>
+      </c>
+      <c r="E23" s="54" t="n">
+        <v>23.48</v>
+      </c>
+      <c r="F23" s="54" t="n">
+        <v>0</v>
+      </c>
       <c r="G23" s="55">
         <f>IF(E23="","",E23-N(F23))</f>
         <v/>
       </c>
-      <c r="H23" s="9" t="n"/>
-      <c r="I23" s="9" t="n"/>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I23" s="9" t="inlineStr">
+        <is>
+          <t>Matches the $23.48 cash expense on Operating Costs — keeps sheet even with bank</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="35" t="n"/>

</xml_diff>